<commit_message>
0.2 - atualizações descritas no README
</commit_message>
<xml_diff>
--- a/resultado_et_hortif.xlsx
+++ b/resultado_et_hortif.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,263 +469,408 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46294</v>
+        <v>46299</v>
       </c>
       <c r="B2" t="n">
-        <v>22.8</v>
+        <v>20.5</v>
       </c>
       <c r="C2" t="n">
-        <v>89.5</v>
+        <v>91.5</v>
       </c>
       <c r="D2" t="n">
-        <v>6.3</v>
+        <v>3.7</v>
       </c>
       <c r="E2" t="n">
-        <v>21.08</v>
+        <v>12.96</v>
       </c>
       <c r="F2" t="n">
-        <v>4.798902798836797</v>
+        <v>3.139601247763712</v>
       </c>
       <c r="G2" t="n">
-        <v>4.32</v>
+        <v>2.83</v>
       </c>
       <c r="H2" t="n">
-        <v>5.04</v>
+        <v>3.3</v>
       </c>
       <c r="I2" t="n">
-        <v>4.56</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="B3" t="n">
-        <v>24.1</v>
+        <v>19.1</v>
       </c>
       <c r="C3" t="n">
-        <v>87</v>
+        <v>89.8</v>
       </c>
       <c r="D3" t="n">
-        <v>5.2</v>
+        <v>7.02</v>
       </c>
       <c r="E3" t="n">
-        <v>18.73</v>
+        <v>7.21</v>
       </c>
       <c r="F3" t="n">
-        <v>4.880832511979006</v>
+        <v>2.012174972961342</v>
       </c>
       <c r="G3" t="n">
-        <v>4.39</v>
+        <v>1.81</v>
       </c>
       <c r="H3" t="n">
-        <v>5.12</v>
+        <v>2.11</v>
       </c>
       <c r="I3" t="n">
-        <v>4.64</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B4" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="C4" t="n">
-        <v>97.5</v>
+        <v>97</v>
       </c>
       <c r="D4" t="n">
-        <v>6.6</v>
+        <v>4.91</v>
       </c>
       <c r="E4" t="n">
-        <v>5.58</v>
+        <v>6.59</v>
       </c>
       <c r="F4" t="n">
-        <v>1.116513494106503</v>
+        <v>1.369382778337876</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>1.23</v>
       </c>
       <c r="H4" t="n">
-        <v>1.17</v>
+        <v>1.44</v>
       </c>
       <c r="I4" t="n">
-        <v>1.06</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>20.6</v>
       </c>
       <c r="C5" t="n">
-        <v>92.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="D5" t="n">
-        <v>8.199999999999999</v>
+        <v>3.57</v>
       </c>
       <c r="E5" t="n">
-        <v>5.83</v>
+        <v>13.91</v>
       </c>
       <c r="F5" t="n">
-        <v>1.481320205782403</v>
+        <v>3.462067214938108</v>
       </c>
       <c r="G5" t="n">
-        <v>1.33</v>
+        <v>3.12</v>
       </c>
       <c r="H5" t="n">
-        <v>1.56</v>
+        <v>3.64</v>
       </c>
       <c r="I5" t="n">
-        <v>1.41</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46298</v>
+        <v>46303</v>
       </c>
       <c r="B6" t="n">
-        <v>20.1</v>
+        <v>22.2</v>
       </c>
       <c r="C6" t="n">
-        <v>85.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>6.21</v>
+        <v>4.16</v>
       </c>
       <c r="E6" t="n">
-        <v>8.970000000000001</v>
+        <v>17.38</v>
       </c>
       <c r="F6" t="n">
-        <v>2.730559905168044</v>
+        <v>4.491296025202758</v>
       </c>
       <c r="G6" t="n">
-        <v>2.46</v>
+        <v>4.04</v>
       </c>
       <c r="H6" t="n">
-        <v>2.87</v>
+        <v>4.72</v>
       </c>
       <c r="I6" t="n">
-        <v>2.59</v>
+        <v>4.27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46299</v>
+        <v>46304</v>
       </c>
       <c r="B7" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="C7" t="n">
-        <v>87</v>
+        <v>87.7</v>
       </c>
       <c r="D7" t="n">
-        <v>3.15</v>
+        <v>4.9</v>
       </c>
       <c r="E7" t="n">
-        <v>17.22</v>
+        <v>16.71</v>
       </c>
       <c r="F7" t="n">
-        <v>4.635478945732509</v>
+        <v>4.348711160008621</v>
       </c>
       <c r="G7" t="n">
-        <v>4.17</v>
+        <v>3.91</v>
       </c>
       <c r="H7" t="n">
-        <v>4.87</v>
+        <v>4.57</v>
       </c>
       <c r="I7" t="n">
-        <v>4.4</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="B8" t="n">
-        <v>19.8</v>
+        <v>23.5</v>
       </c>
       <c r="C8" t="n">
-        <v>92.59999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="D8" t="n">
-        <v>6.44</v>
+        <v>4.82</v>
       </c>
       <c r="E8" t="n">
-        <v>8.609999999999999</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>2.041860700470368</v>
+        <v>2.639142347870003</v>
       </c>
       <c r="G8" t="n">
-        <v>1.84</v>
+        <v>2.38</v>
       </c>
       <c r="H8" t="n">
-        <v>2.14</v>
+        <v>2.77</v>
       </c>
       <c r="I8" t="n">
-        <v>1.94</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="B9" t="n">
-        <v>20.3</v>
+        <v>20.7</v>
       </c>
       <c r="C9" t="n">
-        <v>93.59999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="D9" t="n">
-        <v>4.54</v>
+        <v>6.29</v>
       </c>
       <c r="E9" t="n">
-        <v>13.67</v>
+        <v>5.46</v>
       </c>
       <c r="F9" t="n">
-        <v>3.021698921397299</v>
+        <v>1.165568911713132</v>
       </c>
       <c r="G9" t="n">
-        <v>2.72</v>
+        <v>1.05</v>
       </c>
       <c r="H9" t="n">
-        <v>3.17</v>
+        <v>1.22</v>
       </c>
       <c r="I9" t="n">
-        <v>2.87</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="B10" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="E10" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.149191491739093</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B11" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>92.59999999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.233439636788662</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B12" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="E12" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.287709340796717</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.07</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B13" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.921567960417653</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B14" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="E14" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.829898586440801</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B15" t="n">
         <v>20.3</v>
       </c>
-      <c r="C10" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="D10" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="E10" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2.015412599384489</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="H10" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.91</v>
+      <c r="C15" t="n">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="E15" t="n">
+        <v>20.06</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.92574877296834</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H15" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Alterações nos arquivos de armazenamento dos dados
</commit_message>
<xml_diff>
--- a/resultado_et_hortif.xlsx
+++ b/resultado_et_hortif.xlsx
@@ -469,408 +469,408 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46299</v>
+        <v>46307</v>
       </c>
       <c r="B2" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="C2" t="n">
-        <v>91.5</v>
+        <v>93.3</v>
       </c>
       <c r="D2" t="n">
-        <v>3.7</v>
+        <v>5.09</v>
       </c>
       <c r="E2" t="n">
-        <v>12.96</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>3.139601247763712</v>
+        <v>2.225175589578257</v>
       </c>
       <c r="G2" t="n">
-        <v>2.83</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>3.3</v>
+        <v>2.34</v>
       </c>
       <c r="I2" t="n">
-        <v>2.98</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="B3" t="n">
-        <v>19.1</v>
+        <v>21.1</v>
       </c>
       <c r="C3" t="n">
-        <v>89.8</v>
+        <v>93.8</v>
       </c>
       <c r="D3" t="n">
-        <v>7.02</v>
+        <v>4.68</v>
       </c>
       <c r="E3" t="n">
-        <v>7.21</v>
+        <v>9.27</v>
       </c>
       <c r="F3" t="n">
-        <v>2.012174972961342</v>
+        <v>2.22211344146738</v>
       </c>
       <c r="G3" t="n">
-        <v>1.81</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I3" t="n">
         <v>2.11</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="B4" t="n">
-        <v>18.9</v>
+        <v>21.8</v>
       </c>
       <c r="C4" t="n">
-        <v>97</v>
+        <v>90.5</v>
       </c>
       <c r="D4" t="n">
-        <v>4.91</v>
+        <v>5.41</v>
       </c>
       <c r="E4" t="n">
-        <v>6.59</v>
+        <v>13.77</v>
       </c>
       <c r="F4" t="n">
-        <v>1.369382778337876</v>
+        <v>3.347692729652045</v>
       </c>
       <c r="G4" t="n">
-        <v>1.23</v>
+        <v>3.01</v>
       </c>
       <c r="H4" t="n">
-        <v>1.44</v>
+        <v>3.52</v>
       </c>
       <c r="I4" t="n">
-        <v>1.3</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46302</v>
+        <v>46310</v>
       </c>
       <c r="B5" t="n">
-        <v>20.6</v>
+        <v>23.4</v>
       </c>
       <c r="C5" t="n">
-        <v>89.7</v>
+        <v>86</v>
       </c>
       <c r="D5" t="n">
-        <v>3.57</v>
+        <v>3.9</v>
       </c>
       <c r="E5" t="n">
-        <v>13.91</v>
+        <v>20.54</v>
       </c>
       <c r="F5" t="n">
-        <v>3.462067214938108</v>
+        <v>5.380427740023122</v>
       </c>
       <c r="G5" t="n">
-        <v>3.12</v>
+        <v>4.84</v>
       </c>
       <c r="H5" t="n">
-        <v>3.64</v>
+        <v>5.65</v>
       </c>
       <c r="I5" t="n">
-        <v>3.29</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46303</v>
+        <v>46311</v>
       </c>
       <c r="B6" t="n">
-        <v>22.2</v>
+        <v>22.7</v>
       </c>
       <c r="C6" t="n">
-        <v>86.59999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="D6" t="n">
-        <v>4.16</v>
+        <v>4.96</v>
       </c>
       <c r="E6" t="n">
-        <v>17.38</v>
+        <v>20.98</v>
       </c>
       <c r="F6" t="n">
-        <v>4.491296025202758</v>
+        <v>4.889118273185202</v>
       </c>
       <c r="G6" t="n">
-        <v>4.04</v>
+        <v>4.4</v>
       </c>
       <c r="H6" t="n">
-        <v>4.72</v>
+        <v>5.13</v>
       </c>
       <c r="I6" t="n">
-        <v>4.27</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="B7" t="n">
-        <v>23.3</v>
+        <v>20.7</v>
       </c>
       <c r="C7" t="n">
-        <v>87.7</v>
+        <v>85</v>
       </c>
       <c r="D7" t="n">
-        <v>4.9</v>
+        <v>3.79</v>
       </c>
       <c r="E7" t="n">
-        <v>16.71</v>
+        <v>18.18</v>
       </c>
       <c r="F7" t="n">
-        <v>4.348711160008621</v>
+        <v>4.602025027034761</v>
       </c>
       <c r="G7" t="n">
-        <v>3.91</v>
+        <v>4.14</v>
       </c>
       <c r="H7" t="n">
-        <v>4.57</v>
+        <v>4.83</v>
       </c>
       <c r="I7" t="n">
-        <v>4.13</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46305</v>
+        <v>46313</v>
       </c>
       <c r="B8" t="n">
-        <v>23.5</v>
+        <v>19.7</v>
       </c>
       <c r="C8" t="n">
-        <v>88.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>4.82</v>
+        <v>6.97</v>
       </c>
       <c r="E8" t="n">
-        <v>8.449999999999999</v>
+        <v>23.11</v>
       </c>
       <c r="F8" t="n">
-        <v>2.639142347870003</v>
+        <v>5.654917203712277</v>
       </c>
       <c r="G8" t="n">
-        <v>2.38</v>
+        <v>5.09</v>
       </c>
       <c r="H8" t="n">
-        <v>2.77</v>
+        <v>5.94</v>
       </c>
       <c r="I8" t="n">
-        <v>2.51</v>
+        <v>5.37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46306</v>
+        <v>46314</v>
       </c>
       <c r="B9" t="n">
-        <v>20.7</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>97.3</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>6.29</v>
+        <v>6.26</v>
       </c>
       <c r="E9" t="n">
-        <v>5.46</v>
+        <v>19.17</v>
       </c>
       <c r="F9" t="n">
-        <v>1.165568911713132</v>
+        <v>5.257234391549551</v>
       </c>
       <c r="G9" t="n">
-        <v>1.05</v>
+        <v>4.73</v>
       </c>
       <c r="H9" t="n">
-        <v>1.22</v>
+        <v>5.52</v>
       </c>
       <c r="I9" t="n">
-        <v>1.11</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="B10" t="n">
-        <v>20.4</v>
+        <v>19.1</v>
       </c>
       <c r="C10" t="n">
-        <v>90.8</v>
+        <v>72.2</v>
       </c>
       <c r="D10" t="n">
-        <v>4.65</v>
+        <v>6.33</v>
       </c>
       <c r="E10" t="n">
-        <v>7.94</v>
+        <v>17.7</v>
       </c>
       <c r="F10" t="n">
-        <v>2.149191491739093</v>
+        <v>5.152606940074508</v>
       </c>
       <c r="G10" t="n">
-        <v>1.93</v>
+        <v>4.64</v>
       </c>
       <c r="H10" t="n">
-        <v>2.26</v>
+        <v>5.41</v>
       </c>
       <c r="I10" t="n">
-        <v>2.04</v>
+        <v>4.89</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="B11" t="n">
-        <v>22.4</v>
+        <v>19.6</v>
       </c>
       <c r="C11" t="n">
-        <v>92.59999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="D11" t="n">
-        <v>4.61</v>
+        <v>6.47</v>
       </c>
       <c r="E11" t="n">
-        <v>13.41</v>
+        <v>15</v>
       </c>
       <c r="F11" t="n">
-        <v>3.233439636788662</v>
+        <v>4.180324885103346</v>
       </c>
       <c r="G11" t="n">
-        <v>2.91</v>
+        <v>3.76</v>
       </c>
       <c r="H11" t="n">
-        <v>3.4</v>
+        <v>4.39</v>
       </c>
       <c r="I11" t="n">
-        <v>3.07</v>
+        <v>3.97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="B12" t="n">
-        <v>23.4</v>
+        <v>20.6</v>
       </c>
       <c r="C12" t="n">
-        <v>91.8</v>
+        <v>89.5</v>
       </c>
       <c r="D12" t="n">
-        <v>4.02</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>17.4</v>
+        <v>13.25</v>
       </c>
       <c r="F12" t="n">
-        <v>4.287709340796717</v>
+        <v>3.073844330983777</v>
       </c>
       <c r="G12" t="n">
-        <v>3.86</v>
+        <v>2.77</v>
       </c>
       <c r="H12" t="n">
-        <v>4.5</v>
+        <v>3.23</v>
       </c>
       <c r="I12" t="n">
-        <v>4.07</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="B13" t="n">
-        <v>21.4</v>
+        <v>21</v>
       </c>
       <c r="C13" t="n">
-        <v>91.90000000000001</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>5.7</v>
+        <v>3.53</v>
       </c>
       <c r="E13" t="n">
-        <v>12.39</v>
+        <v>8.01</v>
       </c>
       <c r="F13" t="n">
-        <v>2.921567960417653</v>
+        <v>1.772815608324329</v>
       </c>
       <c r="G13" t="n">
-        <v>2.63</v>
+        <v>1.6</v>
       </c>
       <c r="H13" t="n">
-        <v>3.07</v>
+        <v>1.86</v>
       </c>
       <c r="I13" t="n">
-        <v>2.78</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="B14" t="n">
-        <v>22.1</v>
+        <v>22.7</v>
       </c>
       <c r="C14" t="n">
-        <v>90.3</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>6.87</v>
+        <v>4.72</v>
       </c>
       <c r="E14" t="n">
-        <v>16.9</v>
+        <v>4.68</v>
       </c>
       <c r="F14" t="n">
-        <v>3.829898586440801</v>
+        <v>1.059061818589412</v>
       </c>
       <c r="G14" t="n">
-        <v>3.45</v>
+        <v>0.95</v>
       </c>
       <c r="H14" t="n">
-        <v>4.02</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>3.64</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46312</v>
+        <v>46320</v>
       </c>
       <c r="B15" t="n">
-        <v>20.3</v>
+        <v>22.8</v>
       </c>
       <c r="C15" t="n">
-        <v>80.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>9.82</v>
+        <v>4.68</v>
       </c>
       <c r="E15" t="n">
-        <v>20.06</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>4.92574877296834</v>
+        <v>2.205432870723469</v>
       </c>
       <c r="G15" t="n">
-        <v>4.43</v>
+        <v>1.98</v>
       </c>
       <c r="H15" t="n">
-        <v>5.17</v>
+        <v>2.32</v>
       </c>
       <c r="I15" t="n">
-        <v>4.68</v>
+        <v>2.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Novos arquivos e novas alterações - consultar README
</commit_message>
<xml_diff>
--- a/resultado_et_hortif.xlsx
+++ b/resultado_et_hortif.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,408 +469,263 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="B2" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
       <c r="C2" t="n">
-        <v>93.3</v>
+        <v>69</v>
       </c>
       <c r="D2" t="n">
-        <v>5.09</v>
+        <v>6.13</v>
       </c>
       <c r="E2" t="n">
-        <v>9.539999999999999</v>
+        <v>16.97</v>
       </c>
       <c r="F2" t="n">
-        <v>2.225175589578257</v>
+        <v>5.394710369848077</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>4.86</v>
       </c>
       <c r="H2" t="n">
-        <v>2.34</v>
+        <v>5.66</v>
       </c>
       <c r="I2" t="n">
-        <v>2.11</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="B3" t="n">
-        <v>21.1</v>
+        <v>20.3</v>
       </c>
       <c r="C3" t="n">
-        <v>93.8</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>4.68</v>
+        <v>6.12</v>
       </c>
       <c r="E3" t="n">
-        <v>9.27</v>
+        <v>19.05</v>
       </c>
       <c r="F3" t="n">
-        <v>2.22211344146738</v>
+        <v>5.080668210463539</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>4.57</v>
       </c>
       <c r="H3" t="n">
-        <v>2.33</v>
+        <v>5.33</v>
       </c>
       <c r="I3" t="n">
-        <v>2.11</v>
+        <v>4.83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="B4" t="n">
-        <v>21.8</v>
+        <v>21.2</v>
       </c>
       <c r="C4" t="n">
-        <v>90.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>5.41</v>
+        <v>5.83</v>
       </c>
       <c r="E4" t="n">
-        <v>13.77</v>
+        <v>17.75</v>
       </c>
       <c r="F4" t="n">
-        <v>3.347692729652045</v>
+        <v>4.206020068772324</v>
       </c>
       <c r="G4" t="n">
-        <v>3.01</v>
+        <v>3.79</v>
       </c>
       <c r="H4" t="n">
-        <v>3.52</v>
+        <v>4.42</v>
       </c>
       <c r="I4" t="n">
-        <v>3.18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="B5" t="n">
-        <v>23.4</v>
+        <v>21.4</v>
       </c>
       <c r="C5" t="n">
-        <v>86</v>
+        <v>95.8</v>
       </c>
       <c r="D5" t="n">
-        <v>3.9</v>
+        <v>3.32</v>
       </c>
       <c r="E5" t="n">
-        <v>20.54</v>
+        <v>11.28</v>
       </c>
       <c r="F5" t="n">
-        <v>5.380427740023122</v>
+        <v>2.646663753370305</v>
       </c>
       <c r="G5" t="n">
-        <v>4.84</v>
+        <v>2.38</v>
       </c>
       <c r="H5" t="n">
-        <v>5.65</v>
+        <v>2.78</v>
       </c>
       <c r="I5" t="n">
-        <v>5.11</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="B6" t="n">
-        <v>22.7</v>
+        <v>23.7</v>
       </c>
       <c r="C6" t="n">
-        <v>90.3</v>
+        <v>95.5</v>
       </c>
       <c r="D6" t="n">
-        <v>4.96</v>
+        <v>5.63</v>
       </c>
       <c r="E6" t="n">
-        <v>20.98</v>
+        <v>6.79</v>
       </c>
       <c r="F6" t="n">
-        <v>4.889118273185202</v>
+        <v>1.71357196795594</v>
       </c>
       <c r="G6" t="n">
-        <v>4.4</v>
+        <v>1.54</v>
       </c>
       <c r="H6" t="n">
-        <v>5.13</v>
+        <v>1.8</v>
       </c>
       <c r="I6" t="n">
-        <v>4.64</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46312</v>
+        <v>46320</v>
       </c>
       <c r="B7" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="C7" t="n">
-        <v>85</v>
+        <v>98.7</v>
       </c>
       <c r="D7" t="n">
-        <v>3.79</v>
+        <v>7.24</v>
       </c>
       <c r="E7" t="n">
-        <v>18.18</v>
+        <v>4.58</v>
       </c>
       <c r="F7" t="n">
-        <v>4.602025027034761</v>
+        <v>0.8647418705644474</v>
       </c>
       <c r="G7" t="n">
-        <v>4.14</v>
+        <v>0.78</v>
       </c>
       <c r="H7" t="n">
-        <v>4.83</v>
+        <v>0.91</v>
       </c>
       <c r="I7" t="n">
-        <v>4.37</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46313</v>
+        <v>46321</v>
       </c>
       <c r="B8" t="n">
-        <v>19.7</v>
+        <v>18.7</v>
       </c>
       <c r="C8" t="n">
-        <v>77.59999999999999</v>
+        <v>93.8</v>
       </c>
       <c r="D8" t="n">
-        <v>6.97</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>23.11</v>
+        <v>7.57</v>
       </c>
       <c r="F8" t="n">
-        <v>5.654917203712277</v>
+        <v>1.637120645703077</v>
       </c>
       <c r="G8" t="n">
-        <v>5.09</v>
+        <v>1.47</v>
       </c>
       <c r="H8" t="n">
-        <v>5.94</v>
+        <v>1.72</v>
       </c>
       <c r="I8" t="n">
-        <v>5.37</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46314</v>
+        <v>46322</v>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="C9" t="n">
-        <v>73.59999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>6.26</v>
+        <v>9.07</v>
       </c>
       <c r="E9" t="n">
-        <v>19.17</v>
+        <v>18.55</v>
       </c>
       <c r="F9" t="n">
-        <v>5.257234391549551</v>
+        <v>4.531398402051017</v>
       </c>
       <c r="G9" t="n">
-        <v>4.73</v>
+        <v>4.08</v>
       </c>
       <c r="H9" t="n">
-        <v>5.52</v>
+        <v>4.76</v>
       </c>
       <c r="I9" t="n">
-        <v>4.99</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46315</v>
+        <v>46323</v>
       </c>
       <c r="B10" t="n">
-        <v>19.1</v>
+        <v>21.1</v>
       </c>
       <c r="C10" t="n">
-        <v>72.2</v>
+        <v>78.8</v>
       </c>
       <c r="D10" t="n">
-        <v>6.33</v>
+        <v>6.83</v>
       </c>
       <c r="E10" t="n">
-        <v>17.7</v>
+        <v>13.37</v>
       </c>
       <c r="F10" t="n">
-        <v>5.152606940074508</v>
+        <v>4.203742948798603</v>
       </c>
       <c r="G10" t="n">
-        <v>4.64</v>
+        <v>3.78</v>
       </c>
       <c r="H10" t="n">
-        <v>5.41</v>
+        <v>4.41</v>
       </c>
       <c r="I10" t="n">
-        <v>4.89</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="B11" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="C11" t="n">
-        <v>79.5</v>
-      </c>
-      <c r="D11" t="n">
-        <v>6.47</v>
-      </c>
-      <c r="E11" t="n">
-        <v>15</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.180324885103346</v>
-      </c>
-      <c r="G11" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="H11" t="n">
-        <v>4.39</v>
-      </c>
-      <c r="I11" t="n">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B12" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="C12" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="D12" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="F12" t="n">
-        <v>3.073844330983777</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="H12" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="I12" t="n">
-        <v>2.92</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46318</v>
-      </c>
-      <c r="B13" t="n">
-        <v>21</v>
-      </c>
-      <c r="C13" t="n">
-        <v>98.09999999999999</v>
-      </c>
-      <c r="D13" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="E13" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1.772815608324329</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1.68</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>46319</v>
-      </c>
-      <c r="B14" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="C14" t="n">
-        <v>98.40000000000001</v>
-      </c>
-      <c r="D14" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="E14" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1.059061818589412</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1.01</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46320</v>
-      </c>
-      <c r="B15" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="C15" t="n">
-        <v>94.90000000000001</v>
-      </c>
-      <c r="D15" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="E15" t="n">
-        <v>9.029999999999999</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2.205432870723469</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="H15" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="I15" t="n">
-        <v>2.1</v>
+        <v>3.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>